<commit_message>
Use form for timeline params
</commit_message>
<xml_diff>
--- a/forms/talk-survey/form.xlsx
+++ b/forms/talk-survey/form.xlsx
@@ -1375,7 +1375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="33.5" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1446,6 +1446,11 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>bind::ct:timeline.deleteSources</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>default_language</t>
         </is>
       </c>
@@ -1507,6 +1512,11 @@
         </is>
       </c>
       <c r="L2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>English (en)</t>
         </is>

</xml_diff>